<commit_message>
idk what to write here lol
</commit_message>
<xml_diff>
--- a/data/line_properties.xlsx
+++ b/data/line_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db8d08c81090d50f/Documents/MATLAB/Fill-Simulator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="8_{86C8A9E5-A1D8-4489-A5E0-EA9EDD43E232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F2DF94F-7F70-43AA-AC62-CF9F247B0F66}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="8_{86C8A9E5-A1D8-4489-A5E0-EA9EDD43E232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7AD6B8E-E8E2-4AA9-81A7-8FA1A9D6A281}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FA2D7580-C0BD-4217-ADBF-B96172CDE35E}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t>Parameter</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>ex: "t_pass"</t>
+  </si>
+  <si>
+    <t>Additional Inputs</t>
+  </si>
+  <si>
+    <t>Initial velocity guess (m/s)</t>
   </si>
 </sst>
 </file>
@@ -142,7 +148,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,8 +173,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -284,9 +296,31 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -294,6 +328,19 @@
     </border>
     <border>
       <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="medium">
@@ -302,7 +349,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -311,48 +358,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -368,6 +435,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -690,165 +761,178 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.44140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="18.44140625" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" style="17" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" style="9" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="17.21875" customWidth="1"/>
     <col min="6" max="6" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="16" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="D1" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="19"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15"/>
+      <c r="D2" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="16" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="18"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="D3" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="22"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="7"/>
-    </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="B5" s="4"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="24"/>
+    </row>
+    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="7"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="24"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="25"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="24"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="24"/>
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="24"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+      <c r="B12" s="13"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="24"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="24"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="14" t="s">
+      <c r="B14" s="4"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="24"/>
+    </row>
+    <row r="15" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B15" s="8"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="C1:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
updated excel for line properites
</commit_message>
<xml_diff>
--- a/data/line_properties.xlsx
+++ b/data/line_properties.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emers\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db8d08c81090d50f/Documents/SARP/Fill-Simulator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A41593-C552-44EB-A038-090A3E71F082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{35A41593-C552-44EB-A038-090A3E71F082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00263E9F-A03A-4F43-8E12-D8E39CF521E3}"/>
   <bookViews>
-    <workbookView xWindow="-2385" yWindow="-14505" windowWidth="17280" windowHeight="9960" xr2:uid="{FA2D7580-C0BD-4217-ADBF-B96172CDE35E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FA2D7580-C0BD-4217-ADBF-B96172CDE35E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
   <si>
     <t>Parameter</t>
   </si>
@@ -103,12 +103,6 @@
   </si>
   <si>
     <t>All Fittings on RF Stand</t>
-  </si>
-  <si>
-    <t>Additional Inputs</t>
-  </si>
-  <si>
-    <t>Initial velocity guess (m/s)</t>
   </si>
   <si>
     <t>cross_run</t>
@@ -148,7 +142,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -173,14 +167,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -339,26 +327,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -383,16 +356,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -403,12 +366,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -754,59 +711,42 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.44140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="18.44140625" customWidth="1"/>
     <col min="3" max="3" width="24.109375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="17.21875" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="26" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="25"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="23"/>
+      <c r="B3" s="15"/>
       <c r="C3" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="14"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
@@ -814,12 +754,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="16"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -827,12 +765,10 @@
         <v>0.34645700000000001</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16"/>
-    </row>
-    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -840,12 +776,10 @@
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
@@ -853,20 +787,15 @@
         <v>0.69</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="23"/>
+      <c r="B8" s="15"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
@@ -874,10 +803,8 @@
         <v>2</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -885,10 +812,8 @@
         <v>0.40200000000000002</v>
       </c>
       <c r="C10" s="10"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
-    </row>
-    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
@@ -896,19 +821,15 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="23"/>
+      <c r="B12" s="15"/>
       <c r="C12" s="10"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>6</v>
       </c>
@@ -916,10 +837,8 @@
         <v>30</v>
       </c>
       <c r="C13" s="10"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
@@ -927,10 +846,8 @@
         <v>0.34645700000000001</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
@@ -938,19 +855,16 @@
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="C15" s="10"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D1:E1"/>
     <mergeCell ref="C1:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>